<commit_message>
feat: configure HSRP load balancing and split-scope DHCP across R1 and R2
</commit_message>
<xml_diff>
--- a/Links-n-Addresses.xlsx
+++ b/Links-n-Addresses.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30330"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/cf954df90cd41547/Documents/Cisco-CCNA-200-301/HY-Portfolio/OSPF-Mesh-L2-Distribution/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/cf954df90cd41547/Documents/Cisco-CCNA-200-301/ccna-lab-campus-hsrp/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="596" documentId="11_F25DC773A252ABDACC104804E99B50F05ADE58EA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F46FED8C-0E74-495D-ADBC-1D23299C1C09}"/>
+  <xr:revisionPtr revIDLastSave="814" documentId="11_F25DC773A252ABDACC104804E99B50F05ADE58EA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1388EE67-C196-48B3-9355-7A7051B2D32F}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="441" uniqueCount="149">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="655" uniqueCount="240">
   <si>
     <t>Source</t>
   </si>
@@ -483,6 +484,279 @@
   </si>
   <si>
     <t>NO</t>
+  </si>
+  <si>
+    <t>Upstream</t>
+  </si>
+  <si>
+    <t>Downstream</t>
+  </si>
+  <si>
+    <t>interface gig0/0/0</t>
+  </si>
+  <si>
+    <t>ip address 203.0.113.1 255.255.255.252</t>
+  </si>
+  <si>
+    <t>ipv6 address 2001:db8:0:113::1/64</t>
+  </si>
+  <si>
+    <t>ipv6 fe80::1000 link-local</t>
+  </si>
+  <si>
+    <t>interface gig0/0/1</t>
+  </si>
+  <si>
+    <t>ip address 203.0.114.1 255.255.255.252</t>
+  </si>
+  <si>
+    <t>ipv6 address 2001:db8:0:114::1/64</t>
+  </si>
+  <si>
+    <t>ip address 203.0.113.2 255.255.255.252</t>
+  </si>
+  <si>
+    <t>ipv6 address 2001:db8:0:113::2/64</t>
+  </si>
+  <si>
+    <t>ipv6 fe80::1 link-local</t>
+  </si>
+  <si>
+    <t>interface vlan 100</t>
+  </si>
+  <si>
+    <t>ip address 10.1.0.1 255.255.255.252</t>
+  </si>
+  <si>
+    <t>ipv6 address 2001:db8:0:1::1/64</t>
+  </si>
+  <si>
+    <t>switchport access vlan 100</t>
+  </si>
+  <si>
+    <t>switchport mode access</t>
+  </si>
+  <si>
+    <t>no ip address</t>
+  </si>
+  <si>
+    <t>no ipv6 address</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>interface gig0/0/1.10</t>
+  </si>
+  <si>
+    <t>ip address 192.168.10.1 255.255.255.0</t>
+  </si>
+  <si>
+    <t>ipv6 address 2001:db8:0:10::1/64</t>
+  </si>
+  <si>
+    <t>ipv6 fe80::110 link-local</t>
+  </si>
+  <si>
+    <t>interface gig0/0/1.30</t>
+  </si>
+  <si>
+    <t>interface gig0/0/1.20</t>
+  </si>
+  <si>
+    <t>ip address 192.168.20.1 255.255.255.0</t>
+  </si>
+  <si>
+    <t>ipv6 address 2001:db8:0:20::1/64</t>
+  </si>
+  <si>
+    <t>ip address 192.168.30.1 255.255.255.0</t>
+  </si>
+  <si>
+    <t>ipv6 address 2001:db8:0:30::1/64</t>
+  </si>
+  <si>
+    <t>interface gig0/0/1.900</t>
+  </si>
+  <si>
+    <t>SW1 Vlan 10</t>
+  </si>
+  <si>
+    <t>SW1 Vlan 30</t>
+  </si>
+  <si>
+    <t>SW1 Vlan 20</t>
+  </si>
+  <si>
+    <t>ipv6 address 2001:db8:0:114::2/64</t>
+  </si>
+  <si>
+    <t>ipv6 fe80::2 link-local</t>
+  </si>
+  <si>
+    <t>interface loopback0</t>
+  </si>
+  <si>
+    <t>ip address 10.1.0.2 255.255.255.252</t>
+  </si>
+  <si>
+    <t>ipv6 address 2001:db8:0:1::2/64</t>
+  </si>
+  <si>
+    <t>ip address 192.168.10.2 255.255.255.0</t>
+  </si>
+  <si>
+    <t>ipv6 address 2001:db8:0:10::2/64</t>
+  </si>
+  <si>
+    <t>ipv6 fe80::210 link-local</t>
+  </si>
+  <si>
+    <t>ip address 192.168.20.2 255.255.255.0</t>
+  </si>
+  <si>
+    <t>ipv6 address 2001:db8:0:20::2/64</t>
+  </si>
+  <si>
+    <t>ipv6 fe80::220 link-local</t>
+  </si>
+  <si>
+    <t>ip address 192.168.30.2 255.255.255.0</t>
+  </si>
+  <si>
+    <t>ipv6 address 2001:db8:0:30::2/64</t>
+  </si>
+  <si>
+    <t>ipv6 fe80::230 link-local</t>
+  </si>
+  <si>
+    <t>interface gig0/0/1.99</t>
+  </si>
+  <si>
+    <t>ip address 192.168.99.2 255.255.255.0</t>
+  </si>
+  <si>
+    <t>ipv6 address 2001:db8:0:99::2/64</t>
+  </si>
+  <si>
+    <t>ipv6 fe80::299 link-local</t>
+  </si>
+  <si>
+    <t>ip address 192.168.99.1 255.255.255.0</t>
+  </si>
+  <si>
+    <t>ipv6 address 2001:db8:0:99::1/64</t>
+  </si>
+  <si>
+    <t>ipv6 fe80::199 link-local</t>
+  </si>
+  <si>
+    <t>ipv6 fe80::120 link-local</t>
+  </si>
+  <si>
+    <t>ipv6 fe80::130 link-local</t>
+  </si>
+  <si>
+    <t>ip address 192.168.100.1 255.255.255.255</t>
+  </si>
+  <si>
+    <t>ipv6 address 2001:db8:0:100::1/128</t>
+  </si>
+  <si>
+    <t>ipv6 address 2001:db8:0:100::2/128</t>
+  </si>
+  <si>
+    <t>ip address 192.168.100.2 255.255.255.255</t>
+  </si>
+  <si>
+    <t>interface vlan 99</t>
+  </si>
+  <si>
+    <t>ip address 192.168.99.11 255.255.255.0</t>
+  </si>
+  <si>
+    <t>ipv6 address 2001:db8:0:99::11/64</t>
+  </si>
+  <si>
+    <t>ipv6 fe80::11 link-local</t>
+  </si>
+  <si>
+    <t>interface gig0/1</t>
+  </si>
+  <si>
+    <t>switchport mode trunk</t>
+  </si>
+  <si>
+    <t>switchport trunk native vlan 900</t>
+  </si>
+  <si>
+    <t>switchport trunk allowed vlan 10,20,30,99,900</t>
+  </si>
+  <si>
+    <t>interface gig0/2</t>
+  </si>
+  <si>
+    <t>interface gig0/1/0</t>
+  </si>
+  <si>
+    <t>SW1 Vlan 900</t>
+  </si>
+  <si>
+    <t>SW1 Vlan 99</t>
+  </si>
+  <si>
+    <t>ip address 203.0.114.2 255.255.255.252</t>
+  </si>
+  <si>
+    <t>encapsulation dot1q 900 native</t>
+  </si>
+  <si>
+    <t>encapsulation dot1q 99</t>
+  </si>
+  <si>
+    <t>encapsulation dot1q 10</t>
+  </si>
+  <si>
+    <t>encapsulation dot1q 20</t>
+  </si>
+  <si>
+    <t>encapsulation dot1q 30</t>
+  </si>
+  <si>
+    <t>interface fa0/24</t>
+  </si>
+  <si>
+    <t>switchport trunk allowed vlan 10,20,30,99</t>
+  </si>
+  <si>
+    <t>interface fa0/1</t>
+  </si>
+  <si>
+    <t>interface fa0/2</t>
+  </si>
+  <si>
+    <t>interface fa0/3</t>
+  </si>
+  <si>
+    <t>interface fa0/4</t>
+  </si>
+  <si>
+    <t>ip address 192.168.99.12 255.255.255.0</t>
+  </si>
+  <si>
+    <t>ipv6 address 2001:db8:0:99::12/64</t>
+  </si>
+  <si>
+    <t>ipv6 fe80::12 link-local</t>
+  </si>
+  <si>
+    <t>interface gig0/0/2</t>
+  </si>
+  <si>
+    <t>Un-config-ed on R2</t>
+  </si>
+  <si>
+    <t>Un-config-ed on R1</t>
   </si>
 </sst>
 </file>
@@ -545,6 +819,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2320,4 +2598,740 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B77C65B-01C9-4975-834B-4C3F2F692F62}">
+  <dimension ref="A1:L72"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="19.77734375" customWidth="1"/>
+    <col min="3" max="3" width="23.21875" customWidth="1"/>
+    <col min="4" max="4" width="30.5546875" customWidth="1"/>
+    <col min="5" max="5" width="21.77734375" customWidth="1"/>
+    <col min="9" max="9" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="34" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="29.5546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="21.6640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>149</v>
+      </c>
+      <c r="H1" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>151</v>
+      </c>
+      <c r="C2" t="s">
+        <v>152</v>
+      </c>
+      <c r="D2" t="s">
+        <v>153</v>
+      </c>
+      <c r="E2" t="s">
+        <v>154</v>
+      </c>
+      <c r="H2" t="s">
+        <v>4</v>
+      </c>
+      <c r="I2" t="s">
+        <v>151</v>
+      </c>
+      <c r="J2" t="s">
+        <v>158</v>
+      </c>
+      <c r="K2" t="s">
+        <v>159</v>
+      </c>
+      <c r="L2" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>155</v>
+      </c>
+      <c r="C5" t="s">
+        <v>156</v>
+      </c>
+      <c r="D5" t="s">
+        <v>157</v>
+      </c>
+      <c r="E5" t="s">
+        <v>154</v>
+      </c>
+      <c r="H5" t="s">
+        <v>14</v>
+      </c>
+      <c r="I5" t="s">
+        <v>151</v>
+      </c>
+      <c r="J5" t="s">
+        <v>222</v>
+      </c>
+      <c r="K5" t="s">
+        <v>183</v>
+      </c>
+      <c r="L5" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>4</v>
+      </c>
+      <c r="B9" t="s">
+        <v>161</v>
+      </c>
+      <c r="C9" t="s">
+        <v>162</v>
+      </c>
+      <c r="D9" t="s">
+        <v>163</v>
+      </c>
+      <c r="E9" t="s">
+        <v>160</v>
+      </c>
+      <c r="H9" t="s">
+        <v>14</v>
+      </c>
+      <c r="I9" t="s">
+        <v>161</v>
+      </c>
+      <c r="J9" t="s">
+        <v>186</v>
+      </c>
+      <c r="K9" t="s">
+        <v>187</v>
+      </c>
+      <c r="L9" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="B10" t="s">
+        <v>219</v>
+      </c>
+      <c r="C10" t="s">
+        <v>165</v>
+      </c>
+      <c r="D10" t="s">
+        <v>164</v>
+      </c>
+      <c r="I10" t="s">
+        <v>219</v>
+      </c>
+      <c r="J10" t="s">
+        <v>165</v>
+      </c>
+      <c r="K10" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="B12" t="s">
+        <v>155</v>
+      </c>
+      <c r="C12" t="s">
+        <v>166</v>
+      </c>
+      <c r="D12" t="s">
+        <v>167</v>
+      </c>
+      <c r="E12" t="s">
+        <v>168</v>
+      </c>
+      <c r="H12" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="B13" t="s">
+        <v>169</v>
+      </c>
+      <c r="C13" t="s">
+        <v>170</v>
+      </c>
+      <c r="D13" t="s">
+        <v>171</v>
+      </c>
+      <c r="E13" t="s">
+        <v>172</v>
+      </c>
+      <c r="F13" t="s">
+        <v>225</v>
+      </c>
+      <c r="H13" t="s">
+        <v>180</v>
+      </c>
+      <c r="I13" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="B15" t="s">
+        <v>174</v>
+      </c>
+      <c r="C15" t="s">
+        <v>175</v>
+      </c>
+      <c r="D15" t="s">
+        <v>176</v>
+      </c>
+      <c r="E15" t="s">
+        <v>205</v>
+      </c>
+      <c r="F15" t="s">
+        <v>225</v>
+      </c>
+      <c r="H15" t="s">
+        <v>182</v>
+      </c>
+      <c r="I15" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B17" t="s">
+        <v>173</v>
+      </c>
+      <c r="C17" t="s">
+        <v>177</v>
+      </c>
+      <c r="D17" t="s">
+        <v>178</v>
+      </c>
+      <c r="E17" t="s">
+        <v>204</v>
+      </c>
+      <c r="F17" t="s">
+        <v>226</v>
+      </c>
+      <c r="H17" t="s">
+        <v>181</v>
+      </c>
+      <c r="I17" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B19" t="s">
+        <v>197</v>
+      </c>
+      <c r="C19" t="s">
+        <v>201</v>
+      </c>
+      <c r="D19" t="s">
+        <v>202</v>
+      </c>
+      <c r="E19" t="s">
+        <v>203</v>
+      </c>
+      <c r="F19" t="s">
+        <v>227</v>
+      </c>
+      <c r="H19" t="s">
+        <v>221</v>
+      </c>
+      <c r="I19" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B21" t="s">
+        <v>179</v>
+      </c>
+      <c r="F21" t="s">
+        <v>223</v>
+      </c>
+      <c r="H21" t="s">
+        <v>220</v>
+      </c>
+      <c r="I21" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B23" t="s">
+        <v>185</v>
+      </c>
+      <c r="C23" t="s">
+        <v>206</v>
+      </c>
+      <c r="D23" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>14</v>
+      </c>
+      <c r="B25" t="s">
+        <v>161</v>
+      </c>
+      <c r="C25" t="s">
+        <v>186</v>
+      </c>
+      <c r="D25" t="s">
+        <v>187</v>
+      </c>
+      <c r="E25" t="s">
+        <v>184</v>
+      </c>
+      <c r="H25" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B26" t="s">
+        <v>219</v>
+      </c>
+      <c r="C26" t="s">
+        <v>165</v>
+      </c>
+      <c r="D26" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B28" t="s">
+        <v>155</v>
+      </c>
+      <c r="C28" t="s">
+        <v>166</v>
+      </c>
+      <c r="D28" t="s">
+        <v>167</v>
+      </c>
+      <c r="E28" t="s">
+        <v>168</v>
+      </c>
+      <c r="H28" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B29" t="s">
+        <v>169</v>
+      </c>
+      <c r="C29" t="s">
+        <v>188</v>
+      </c>
+      <c r="D29" t="s">
+        <v>189</v>
+      </c>
+      <c r="E29" t="s">
+        <v>190</v>
+      </c>
+      <c r="F29" t="s">
+        <v>225</v>
+      </c>
+      <c r="H29" t="s">
+        <v>180</v>
+      </c>
+      <c r="I29" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B31" t="s">
+        <v>174</v>
+      </c>
+      <c r="C31" t="s">
+        <v>191</v>
+      </c>
+      <c r="D31" t="s">
+        <v>192</v>
+      </c>
+      <c r="E31" t="s">
+        <v>193</v>
+      </c>
+      <c r="F31" t="s">
+        <v>226</v>
+      </c>
+      <c r="H31" t="s">
+        <v>182</v>
+      </c>
+      <c r="I31" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B33" t="s">
+        <v>173</v>
+      </c>
+      <c r="C33" t="s">
+        <v>194</v>
+      </c>
+      <c r="D33" t="s">
+        <v>195</v>
+      </c>
+      <c r="E33" t="s">
+        <v>196</v>
+      </c>
+      <c r="F33" t="s">
+        <v>227</v>
+      </c>
+      <c r="H33" t="s">
+        <v>181</v>
+      </c>
+      <c r="I33" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B35" t="s">
+        <v>197</v>
+      </c>
+      <c r="C35" t="s">
+        <v>198</v>
+      </c>
+      <c r="D35" t="s">
+        <v>199</v>
+      </c>
+      <c r="E35" t="s">
+        <v>200</v>
+      </c>
+      <c r="F35" t="s">
+        <v>224</v>
+      </c>
+      <c r="I35" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B37" t="s">
+        <v>179</v>
+      </c>
+      <c r="F37" t="s">
+        <v>223</v>
+      </c>
+      <c r="I37" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B39" t="s">
+        <v>185</v>
+      </c>
+      <c r="C39" t="s">
+        <v>209</v>
+      </c>
+      <c r="D39" t="s">
+        <v>208</v>
+      </c>
+      <c r="E39" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>26</v>
+      </c>
+      <c r="B41" t="s">
+        <v>210</v>
+      </c>
+      <c r="C41" t="s">
+        <v>211</v>
+      </c>
+      <c r="D41" t="s">
+        <v>212</v>
+      </c>
+      <c r="E41" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B43" t="s">
+        <v>214</v>
+      </c>
+      <c r="C43" t="s">
+        <v>215</v>
+      </c>
+      <c r="D43" t="s">
+        <v>216</v>
+      </c>
+      <c r="E43" t="s">
+        <v>217</v>
+      </c>
+      <c r="H43" t="s">
+        <v>4</v>
+      </c>
+      <c r="I43" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B45" t="s">
+        <v>218</v>
+      </c>
+      <c r="C45" t="s">
+        <v>215</v>
+      </c>
+      <c r="D45" t="s">
+        <v>216</v>
+      </c>
+      <c r="E45" t="s">
+        <v>217</v>
+      </c>
+      <c r="H45" t="s">
+        <v>14</v>
+      </c>
+      <c r="I45" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B47" t="s">
+        <v>228</v>
+      </c>
+      <c r="C47" t="s">
+        <v>215</v>
+      </c>
+      <c r="D47" t="s">
+        <v>216</v>
+      </c>
+      <c r="E47" t="s">
+        <v>229</v>
+      </c>
+      <c r="H47" t="s">
+        <v>27</v>
+      </c>
+      <c r="I47" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="49" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="B49" t="s">
+        <v>230</v>
+      </c>
+      <c r="C49" t="s">
+        <v>215</v>
+      </c>
+      <c r="D49" t="s">
+        <v>216</v>
+      </c>
+      <c r="E49" t="s">
+        <v>229</v>
+      </c>
+      <c r="H49" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="51" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="B51" t="s">
+        <v>231</v>
+      </c>
+      <c r="C51" t="s">
+        <v>215</v>
+      </c>
+      <c r="D51" t="s">
+        <v>216</v>
+      </c>
+      <c r="E51" t="s">
+        <v>229</v>
+      </c>
+      <c r="H51" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="53" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="B53" t="s">
+        <v>232</v>
+      </c>
+      <c r="C53" t="s">
+        <v>215</v>
+      </c>
+      <c r="D53" t="s">
+        <v>216</v>
+      </c>
+      <c r="E53" t="s">
+        <v>229</v>
+      </c>
+      <c r="H53" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="55" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="B55" t="s">
+        <v>233</v>
+      </c>
+      <c r="C55" t="s">
+        <v>215</v>
+      </c>
+      <c r="D55" t="s">
+        <v>216</v>
+      </c>
+      <c r="E55" t="s">
+        <v>229</v>
+      </c>
+      <c r="H55" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="58" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A58" t="s">
+        <v>27</v>
+      </c>
+      <c r="B58" t="s">
+        <v>210</v>
+      </c>
+      <c r="C58" t="s">
+        <v>234</v>
+      </c>
+      <c r="D58" t="s">
+        <v>235</v>
+      </c>
+      <c r="E58" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="60" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="B60" t="s">
+        <v>214</v>
+      </c>
+      <c r="C60" t="s">
+        <v>215</v>
+      </c>
+      <c r="D60" t="s">
+        <v>216</v>
+      </c>
+      <c r="E60" t="s">
+        <v>229</v>
+      </c>
+      <c r="H60" t="s">
+        <v>4</v>
+      </c>
+      <c r="I60" t="s">
+        <v>237</v>
+      </c>
+      <c r="J60" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="62" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="B62" t="s">
+        <v>218</v>
+      </c>
+      <c r="C62" t="s">
+        <v>215</v>
+      </c>
+      <c r="D62" t="s">
+        <v>216</v>
+      </c>
+      <c r="E62" t="s">
+        <v>229</v>
+      </c>
+      <c r="H62" t="s">
+        <v>14</v>
+      </c>
+      <c r="I62" t="s">
+        <v>237</v>
+      </c>
+      <c r="J62" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="64" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="B64" t="s">
+        <v>228</v>
+      </c>
+      <c r="C64" t="s">
+        <v>215</v>
+      </c>
+      <c r="D64" t="s">
+        <v>216</v>
+      </c>
+      <c r="E64" t="s">
+        <v>229</v>
+      </c>
+      <c r="H64" t="s">
+        <v>26</v>
+      </c>
+      <c r="I64" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="66" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B66" t="s">
+        <v>230</v>
+      </c>
+      <c r="C66" t="s">
+        <v>215</v>
+      </c>
+      <c r="D66" t="s">
+        <v>216</v>
+      </c>
+      <c r="E66" t="s">
+        <v>229</v>
+      </c>
+      <c r="H66" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="68" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B68" t="s">
+        <v>231</v>
+      </c>
+      <c r="C68" t="s">
+        <v>215</v>
+      </c>
+      <c r="D68" t="s">
+        <v>216</v>
+      </c>
+      <c r="E68" t="s">
+        <v>229</v>
+      </c>
+      <c r="H68" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="70" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B70" t="s">
+        <v>232</v>
+      </c>
+      <c r="C70" t="s">
+        <v>215</v>
+      </c>
+      <c r="D70" t="s">
+        <v>216</v>
+      </c>
+      <c r="E70" t="s">
+        <v>229</v>
+      </c>
+      <c r="H70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="72" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B72" t="s">
+        <v>233</v>
+      </c>
+      <c r="C72" t="s">
+        <v>215</v>
+      </c>
+      <c r="D72" t="s">
+        <v>216</v>
+      </c>
+      <c r="E72" t="s">
+        <v>229</v>
+      </c>
+      <c r="H72" t="s">
+        <v>34</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: configure OSPF Area 0 dynamic routing and default route failover across R1 and R2
</commit_message>
<xml_diff>
--- a/Links-n-Addresses.xlsx
+++ b/Links-n-Addresses.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/cf954df90cd41547/Documents/Cisco-CCNA-200-301/ccna-lab-campus-hsrp/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="814" documentId="11_F25DC773A252ABDACC104804E99B50F05ADE58EA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1388EE67-C196-48B3-9355-7A7051B2D32F}"/>
+  <xr:revisionPtr revIDLastSave="847" documentId="11_F25DC773A252ABDACC104804E99B50F05ADE58EA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{09483EF0-743E-4047-B10B-61A7D222D72A}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="655" uniqueCount="240">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="683" uniqueCount="252">
   <si>
     <t>Source</t>
   </si>
@@ -757,6 +757,42 @@
   </si>
   <si>
     <t>Un-config-ed on R1</t>
+  </si>
+  <si>
+    <t>ip address 192.168.99.32 255.255.255.0</t>
+  </si>
+  <si>
+    <t>ipv6 address 2001:db8:0:99::32/64</t>
+  </si>
+  <si>
+    <t>ipv6 fe80::32 link-local</t>
+  </si>
+  <si>
+    <t>ip address 192.168.99.33 255.255.255.0</t>
+  </si>
+  <si>
+    <t>ipv6 address 2001:db8:0:99::33/64</t>
+  </si>
+  <si>
+    <t>ipv6 fe80::33 link-local</t>
+  </si>
+  <si>
+    <t>ip address 192.168.99.34 255.255.255.0</t>
+  </si>
+  <si>
+    <t>ipv6 address 2001:db8:0:99::34/64</t>
+  </si>
+  <si>
+    <t>ipv6 fe80::34 link-local</t>
+  </si>
+  <si>
+    <t>ip address 192.168.99.36 255.255.255.0</t>
+  </si>
+  <si>
+    <t>ipv6 address 2001:db8:0:99::36/64</t>
+  </si>
+  <si>
+    <t>ipv6 fe80::36 link-local</t>
   </si>
 </sst>
 </file>
@@ -2602,13 +2638,15 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B77C65B-01C9-4975-834B-4C3F2F692F62}">
-  <dimension ref="A1:L72"/>
+  <dimension ref="A1:L90"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="19.77734375" customWidth="1"/>
     <col min="3" max="3" width="23.21875" customWidth="1"/>
     <col min="4" max="4" width="30.5546875" customWidth="1"/>
     <col min="5" max="5" width="21.77734375" customWidth="1"/>
+    <col min="7" max="7" width="15.33203125" customWidth="1"/>
+    <col min="8" max="8" width="14.5546875" customWidth="1"/>
     <col min="9" max="9" width="15.6640625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="34" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="29.5546875" bestFit="1" customWidth="1"/>
@@ -3128,6 +3166,9 @@
       <c r="H49" t="s">
         <v>31</v>
       </c>
+      <c r="I49" t="s">
+        <v>230</v>
+      </c>
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B51" t="s">
@@ -3145,6 +3186,9 @@
       <c r="H51" t="s">
         <v>32</v>
       </c>
+      <c r="I51" t="s">
+        <v>230</v>
+      </c>
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B53" t="s">
@@ -3162,6 +3206,9 @@
       <c r="H53" t="s">
         <v>33</v>
       </c>
+      <c r="I53" t="s">
+        <v>230</v>
+      </c>
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B55" t="s">
@@ -3179,6 +3226,9 @@
       <c r="H55" t="s">
         <v>34</v>
       </c>
+      <c r="I55" t="s">
+        <v>230</v>
+      </c>
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
@@ -3263,7 +3313,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="66" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B66" t="s">
         <v>230</v>
       </c>
@@ -3279,8 +3329,11 @@
       <c r="H66" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="68" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I66" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="68" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B68" t="s">
         <v>231</v>
       </c>
@@ -3296,8 +3349,11 @@
       <c r="H68" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="70" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I68" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="70" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B70" t="s">
         <v>232</v>
       </c>
@@ -3313,8 +3369,11 @@
       <c r="H70" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="72" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I70" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="72" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B72" t="s">
         <v>233</v>
       </c>
@@ -3329,6 +3388,77 @@
       </c>
       <c r="H72" t="s">
         <v>34</v>
+      </c>
+      <c r="I72" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="75" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A75" t="s">
+        <v>31</v>
+      </c>
+      <c r="B75" t="s">
+        <v>210</v>
+      </c>
+      <c r="C75" t="s">
+        <v>240</v>
+      </c>
+      <c r="D75" t="s">
+        <v>241</v>
+      </c>
+      <c r="E75" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="80" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A80" t="s">
+        <v>32</v>
+      </c>
+      <c r="B80" t="s">
+        <v>210</v>
+      </c>
+      <c r="C80" t="s">
+        <v>243</v>
+      </c>
+      <c r="D80" t="s">
+        <v>244</v>
+      </c>
+      <c r="E80" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A85" t="s">
+        <v>33</v>
+      </c>
+      <c r="B85" t="s">
+        <v>210</v>
+      </c>
+      <c r="C85" t="s">
+        <v>246</v>
+      </c>
+      <c r="D85" t="s">
+        <v>247</v>
+      </c>
+      <c r="E85" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="90" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A90" t="s">
+        <v>32</v>
+      </c>
+      <c r="B90" t="s">
+        <v>210</v>
+      </c>
+      <c r="C90" t="s">
+        <v>249</v>
+      </c>
+      <c r="D90" t="s">
+        <v>250</v>
+      </c>
+      <c r="E90" t="s">
+        <v>251</v>
       </c>
     </row>
   </sheetData>

</xml_diff>